<commit_message>
Correct the Hein et al. 2006 curation and refit affected parameters (v1.1.0)
Hein et al. 2006 (SR17): its k_on,G and K_d were 1/(tau_on x 1 mM agonist).
tau_on was measured at saturating agonist and no G-protein concentration is
reported, so both were removed; its k_off,G values are unchanged. Its Gs
activation and deactivation time constants (Fig. 2) were added to k_act and
k_inact.

- data: both curated workbooks and GPCR_parameters.xlsx.
- BHM: Kd, konG, kact and kinact refit; all other parameters keep their
  2026-09-24 fits.
- REM: k_act and k_inact refit; k_inact forest-plot axis widened.
- Tables S5 and S6, Figure S17, the K_d check, Figures 3-5 regenerated.
- Figure 1 re-exported with the new intervals; Figure 2 BioRender credit.
- README: pooled estimates, version history, citation.
</commit_message>
<xml_diff>
--- a/data/GPCR_parameters.xlsx
+++ b/data/GPCR_parameters.xlsx
@@ -1384,13 +1384,13 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>1900</v>
+        <v>863</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>253</v>
+        <v>18.6</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>5590</v>
+        <v>3090</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -1415,13 +1415,13 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>1820000</v>
+        <v>3150000</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>104000</v>
+        <v>134000</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>5650000</v>
+        <v>12000000</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -1477,22 +1477,22 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>3.27</v>
+        <v>4.59</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.8080000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>7.44</v>
+        <v>10.6</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>24.8</v>
+        <v>30.4</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>9.66</v>
+        <v>12.8</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>63.5</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="6">
@@ -1502,22 +1502,22 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>1.81</v>
+        <v>2.04</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0.117</v>
+        <v>0.302</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>5.82</v>
+        <v>5.2</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>14</v>
+        <v>7.02</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>11.5</v>
+        <v>2.87</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="7">
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>1820000</v>
+        <v>3150000</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>104000</v>
+        <v>134000</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>5650000</v>
+        <v>12000000</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -1875,22 +1875,22 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>3.27</v>
+        <v>4.59</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.8080000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>7.44</v>
+        <v>10.6</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>24.8</v>
+        <v>30.4</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>9.66</v>
+        <v>12.8</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>63.5</v>
+        <v>72.3</v>
       </c>
       <c r="H4" s="4" t="n"/>
     </row>
@@ -1901,22 +1901,22 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>1.81</v>
+        <v>2.04</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.117</v>
+        <v>0.302</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>5.82</v>
+        <v>5.2</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>14</v>
+        <v>7.02</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>11.5</v>
+        <v>2.87</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="H5" s="4" t="n"/>
     </row>
@@ -2366,10 +2366,10 @@
         </is>
       </c>
       <c r="B2" s="25" t="n">
-        <v>3.21864</v>
+        <v>3.107548</v>
       </c>
       <c r="C2" s="25" t="n">
-        <v>22401.8</v>
+        <v>22932.0547</v>
       </c>
       <c r="D2" s="30" t="n">
         <v>100</v>
@@ -2399,10 +2399,10 @@
         </is>
       </c>
       <c r="B3" s="25" t="n">
-        <v>3.07692</v>
+        <v>2.882423</v>
       </c>
       <c r="C3" s="25" t="n">
-        <v>4242</v>
+        <v>3328.2925</v>
       </c>
       <c r="D3" s="30" t="n">
         <v>100</v>
@@ -2432,25 +2432,25 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>0.019092</v>
+        <v>1.02011</v>
       </c>
       <c r="C4" s="25" t="n">
-        <v>5.8729</v>
+        <v>1234.6346</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>0.0530538</v>
+        <v>4.93992e-266</v>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>NS</t>
+          <t>***</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Substantial</t>
+          <t>Extreme</t>
         </is>
       </c>
       <c r="H4" s="19" t="n"/>
@@ -2981,7 +2981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -4397,46 +4397,38 @@
       <c r="G67" s="38" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="35" t="inlineStr">
-        <is>
-          <t>Kba</t>
+      <c r="A68" s="36" t="inlineStr">
+        <is>
+          <t>Kact, Kinact</t>
         </is>
       </c>
       <c r="B68" s="32" t="inlineStr">
         <is>
-          <t>OXTR</t>
+          <t>A2AR</t>
         </is>
       </c>
       <c r="C68" s="32" t="inlineStr">
         <is>
-          <t>oxytocin</t>
-        </is>
-      </c>
-      <c r="D68" s="38" t="n"/>
-      <c r="E68" s="38" t="n"/>
-      <c r="F68" s="38" t="n"/>
-      <c r="G68" s="38" t="n"/>
+          <t>adenosine</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="35" t="inlineStr">
-        <is>
-          <t>Kba</t>
+      <c r="A69" s="36" t="inlineStr">
+        <is>
+          <t>Kact, Kinact</t>
         </is>
       </c>
       <c r="B69" s="32" t="inlineStr">
         <is>
-          <t>OXTR</t>
+          <t>β1AR</t>
         </is>
       </c>
       <c r="C69" s="32" t="inlineStr">
         <is>
-          <t>oxytocin</t>
-        </is>
-      </c>
-      <c r="D69" s="38" t="n"/>
-      <c r="E69" s="38" t="n"/>
-      <c r="F69" s="38" t="n"/>
-      <c r="G69" s="38" t="n"/>
+          <t>norepinephrine</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
@@ -4530,12 +4522,12 @@
       </c>
       <c r="B74" s="32" t="inlineStr">
         <is>
-          <t>V2R</t>
+          <t>OXTR</t>
         </is>
       </c>
       <c r="C74" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t>oxytocin</t>
         </is>
       </c>
       <c r="D74" s="38" t="n"/>
@@ -4551,12 +4543,12 @@
       </c>
       <c r="B75" s="32" t="inlineStr">
         <is>
-          <t>V2R</t>
+          <t>OXTR</t>
         </is>
       </c>
       <c r="C75" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t>oxytocin</t>
         </is>
       </c>
       <c r="D75" s="38" t="n"/>
@@ -4572,12 +4564,12 @@
       </c>
       <c r="B76" s="32" t="inlineStr">
         <is>
-          <t>AT1R</t>
+          <t>V2R</t>
         </is>
       </c>
       <c r="C76" s="32" t="inlineStr">
         <is>
-          <t>angiotensin II</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D76" s="38" t="n"/>
@@ -4593,12 +4585,12 @@
       </c>
       <c r="B77" s="32" t="inlineStr">
         <is>
-          <t>AT1R</t>
+          <t>V2R</t>
         </is>
       </c>
       <c r="C77" s="32" t="inlineStr">
         <is>
-          <t>angiotensin II</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D77" s="38" t="n"/>
@@ -4656,12 +4648,12 @@
       </c>
       <c r="B80" s="32" t="inlineStr">
         <is>
-          <t>β2AR</t>
+          <t>AT1R</t>
         </is>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
-          <t>isoproterenol</t>
+          <t>angiotensin II</t>
         </is>
       </c>
       <c r="D80" s="38" t="n"/>
@@ -4677,12 +4669,12 @@
       </c>
       <c r="B81" s="32" t="inlineStr">
         <is>
-          <t>β2AR</t>
+          <t>AT1R</t>
         </is>
       </c>
       <c r="C81" s="32" t="inlineStr">
         <is>
-          <t>isoproterenol</t>
+          <t>angiotensin II</t>
         </is>
       </c>
       <c r="D81" s="38" t="n"/>
@@ -4735,17 +4727,17 @@
     <row r="84">
       <c r="A84" s="35" t="inlineStr">
         <is>
-          <t>Kint</t>
+          <t>Kba</t>
         </is>
       </c>
       <c r="B84" s="32" t="inlineStr">
         <is>
-          <t>OXTR</t>
+          <t>β2AR</t>
         </is>
       </c>
       <c r="C84" s="32" t="inlineStr">
         <is>
-          <t>oxytocin</t>
+          <t>isoproterenol</t>
         </is>
       </c>
       <c r="D84" s="38" t="n"/>
@@ -4756,17 +4748,17 @@
     <row r="85">
       <c r="A85" s="35" t="inlineStr">
         <is>
-          <t>Kint</t>
+          <t>Kba</t>
         </is>
       </c>
       <c r="B85" s="32" t="inlineStr">
         <is>
-          <t>OXTR</t>
+          <t>β2AR</t>
         </is>
       </c>
       <c r="C85" s="32" t="inlineStr">
         <is>
-          <t>oxytocin</t>
+          <t>isoproterenol</t>
         </is>
       </c>
       <c r="D85" s="38" t="n"/>
@@ -4782,12 +4774,12 @@
       </c>
       <c r="B86" s="32" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>OXTR</t>
         </is>
       </c>
       <c r="C86" s="32" t="inlineStr">
         <is>
-          <t>human chorionic gonadotropin</t>
+          <t>oxytocin</t>
         </is>
       </c>
       <c r="D86" s="38" t="n"/>
@@ -4803,12 +4795,12 @@
       </c>
       <c r="B87" s="32" t="inlineStr">
         <is>
-          <t>V1R</t>
+          <t>OXTR</t>
         </is>
       </c>
       <c r="C87" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t>oxytocin</t>
         </is>
       </c>
       <c r="D87" s="38" t="n"/>
@@ -4824,12 +4816,12 @@
       </c>
       <c r="B88" s="32" t="inlineStr">
         <is>
-          <t>V2R</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C88" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t>human chorionic gonadotropin</t>
         </is>
       </c>
       <c r="D88" s="38" t="n"/>
@@ -4887,12 +4879,12 @@
       </c>
       <c r="B91" s="32" t="inlineStr">
         <is>
-          <t>CXCR7</t>
+          <t>V1R</t>
         </is>
       </c>
       <c r="C91" s="32" t="inlineStr">
         <is>
-          <t>SR49059</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D91" s="38" t="n"/>
@@ -4906,14 +4898,14 @@
           <t>Kint</t>
         </is>
       </c>
-      <c r="B92" s="37" t="inlineStr">
-        <is>
-          <t>CXCR4</t>
+      <c r="B92" s="32" t="inlineStr">
+        <is>
+          <t>V2R</t>
         </is>
       </c>
       <c r="C92" s="32" t="inlineStr">
         <is>
-          <t>CXCL12</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D92" s="38" t="n"/>
@@ -4927,14 +4919,14 @@
           <t>Kint</t>
         </is>
       </c>
-      <c r="B93" s="37" t="inlineStr">
-        <is>
-          <t>V1AR</t>
+      <c r="B93" s="32" t="inlineStr">
+        <is>
+          <t>CXCR7</t>
         </is>
       </c>
       <c r="C93" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t>SR49059</t>
         </is>
       </c>
       <c r="D93" s="38" t="n"/>
@@ -4948,14 +4940,14 @@
           <t>Kint</t>
         </is>
       </c>
-      <c r="B94" s="32" t="inlineStr">
-        <is>
-          <t>M2R</t>
+      <c r="B94" s="37" t="inlineStr">
+        <is>
+          <t>CXCR4</t>
         </is>
       </c>
       <c r="C94" s="32" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t>CXCL12</t>
         </is>
       </c>
       <c r="D94" s="38" t="n"/>
@@ -4969,14 +4961,14 @@
           <t>Kint</t>
         </is>
       </c>
-      <c r="B95" s="32" t="inlineStr">
-        <is>
-          <t>β2AR</t>
+      <c r="B95" s="37" t="inlineStr">
+        <is>
+          <t>V1AR</t>
         </is>
       </c>
       <c r="C95" s="32" t="inlineStr">
         <is>
-          <t>isoproterenol</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D95" s="38" t="n"/>
@@ -4987,42 +4979,42 @@
     <row r="96">
       <c r="A96" s="35" t="inlineStr">
         <is>
-          <t>Kcons_int</t>
+          <t>Kint</t>
         </is>
       </c>
       <c r="B96" s="32" t="inlineStr">
         <is>
-          <t>M3R</t>
-        </is>
-      </c>
-      <c r="C96" s="34" t="inlineStr">
-        <is>
-          <t>carbachol</t>
-        </is>
-      </c>
-      <c r="D96" s="39" t="n"/>
-      <c r="E96" s="39" t="n"/>
+          <t>M2R</t>
+        </is>
+      </c>
+      <c r="C96" s="32" t="inlineStr">
+        <is>
+          <t>acetylcholine</t>
+        </is>
+      </c>
+      <c r="D96" s="38" t="n"/>
+      <c r="E96" s="38" t="n"/>
       <c r="F96" s="38" t="n"/>
       <c r="G96" s="38" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="35" t="inlineStr">
         <is>
-          <t>Kcons_int</t>
+          <t>Kint</t>
         </is>
       </c>
       <c r="B97" s="32" t="inlineStr">
         <is>
-          <t>CXCR7</t>
+          <t>β2AR</t>
         </is>
       </c>
       <c r="C97" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">CXCL12 </t>
-        </is>
-      </c>
-      <c r="D97" s="39" t="n"/>
-      <c r="E97" s="39" t="n"/>
+          <t>isoproterenol</t>
+        </is>
+      </c>
+      <c r="D97" s="38" t="n"/>
+      <c r="E97" s="38" t="n"/>
       <c r="F97" s="38" t="n"/>
       <c r="G97" s="38" t="n"/>
     </row>
@@ -5034,12 +5026,12 @@
       </c>
       <c r="B98" s="32" t="inlineStr">
         <is>
-          <t>M2R</t>
+          <t>M3R</t>
         </is>
       </c>
       <c r="C98" s="34" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t>carbachol</t>
         </is>
       </c>
       <c r="D98" s="39" t="n"/>
@@ -5055,12 +5047,12 @@
       </c>
       <c r="B99" s="32" t="inlineStr">
         <is>
-          <t>PAR1</t>
-        </is>
-      </c>
-      <c r="C99" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SFLLRN </t>
+          <t>CXCR7</t>
+        </is>
+      </c>
+      <c r="C99" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CXCL12 </t>
         </is>
       </c>
       <c r="D99" s="39" t="n"/>
@@ -5076,12 +5068,12 @@
       </c>
       <c r="B100" s="32" t="inlineStr">
         <is>
-          <t>CXCR4</t>
+          <t>M2R</t>
         </is>
       </c>
       <c r="C100" s="34" t="inlineStr">
         <is>
-          <t>CCL5/CXCL12</t>
+          <t>acetylcholine</t>
         </is>
       </c>
       <c r="D100" s="39" t="n"/>
@@ -5097,12 +5089,12 @@
       </c>
       <c r="B101" s="32" t="inlineStr">
         <is>
-          <t>CXCR5</t>
+          <t>PAR1</t>
         </is>
       </c>
       <c r="C101" s="34" t="inlineStr">
         <is>
-          <t>CCL5/CXCL12</t>
+          <t xml:space="preserve">SFLLRN </t>
         </is>
       </c>
       <c r="D101" s="39" t="n"/>
@@ -5113,17 +5105,17 @@
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
         <is>
-          <t>Krec</t>
+          <t>Kcons_int</t>
         </is>
       </c>
       <c r="B102" s="32" t="inlineStr">
         <is>
-          <t>OXTR</t>
-        </is>
-      </c>
-      <c r="C102" s="32" t="inlineStr">
-        <is>
-          <t>oxytocin</t>
+          <t>CXCR4</t>
+        </is>
+      </c>
+      <c r="C102" s="34" t="inlineStr">
+        <is>
+          <t>CCL5/CXCL12</t>
         </is>
       </c>
       <c r="D102" s="39" t="n"/>
@@ -5134,17 +5126,17 @@
     <row r="103">
       <c r="A103" s="35" t="inlineStr">
         <is>
-          <t>Krec</t>
+          <t>Kcons_int</t>
         </is>
       </c>
       <c r="B103" s="32" t="inlineStr">
         <is>
-          <t>P2Y12R</t>
-        </is>
-      </c>
-      <c r="C103" s="32" t="inlineStr">
-        <is>
-          <t>adenosine diphosphate</t>
+          <t>CXCR5</t>
+        </is>
+      </c>
+      <c r="C103" s="34" t="inlineStr">
+        <is>
+          <t>CCL5/CXCL12</t>
         </is>
       </c>
       <c r="D103" s="39" t="n"/>
@@ -5160,16 +5152,16 @@
       </c>
       <c r="B104" s="32" t="inlineStr">
         <is>
-          <t>P2Y1R</t>
+          <t>OXTR</t>
         </is>
       </c>
       <c r="C104" s="32" t="inlineStr">
         <is>
-          <t>adenosine diphosphate</t>
-        </is>
-      </c>
-      <c r="D104" s="38" t="n"/>
-      <c r="E104" s="38" t="n"/>
+          <t>oxytocin</t>
+        </is>
+      </c>
+      <c r="D104" s="39" t="n"/>
+      <c r="E104" s="39" t="n"/>
       <c r="F104" s="38" t="n"/>
       <c r="G104" s="38" t="n"/>
     </row>
@@ -5181,16 +5173,16 @@
       </c>
       <c r="B105" s="32" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>P2Y12R</t>
         </is>
       </c>
       <c r="C105" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">human chorionic gonadotropin </t>
-        </is>
-      </c>
-      <c r="D105" s="38" t="n"/>
-      <c r="E105" s="38" t="n"/>
+          <t>adenosine diphosphate</t>
+        </is>
+      </c>
+      <c r="D105" s="39" t="n"/>
+      <c r="E105" s="39" t="n"/>
       <c r="F105" s="38" t="n"/>
       <c r="G105" s="38" t="n"/>
     </row>
@@ -5202,12 +5194,12 @@
       </c>
       <c r="B106" s="32" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>P2Y1R</t>
         </is>
       </c>
       <c r="C106" s="32" t="inlineStr">
         <is>
-          <t>transferrin</t>
+          <t>adenosine diphosphate</t>
         </is>
       </c>
       <c r="D106" s="38" t="n"/>
@@ -5223,12 +5215,12 @@
       </c>
       <c r="B107" s="32" t="inlineStr">
         <is>
-          <t>CXCR7</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C107" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">CXCL12 </t>
+          <t xml:space="preserve">human chorionic gonadotropin </t>
         </is>
       </c>
       <c r="D107" s="38" t="n"/>
@@ -5244,12 +5236,12 @@
       </c>
       <c r="B108" s="32" t="inlineStr">
         <is>
-          <t>M2R</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C108" s="32" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t>transferrin</t>
         </is>
       </c>
       <c r="D108" s="38" t="n"/>
@@ -5265,12 +5257,12 @@
       </c>
       <c r="B109" s="32" t="inlineStr">
         <is>
-          <t>V1R</t>
+          <t>CXCR7</t>
         </is>
       </c>
       <c r="C109" s="32" t="inlineStr">
         <is>
-          <t>arginine vasopressin</t>
+          <t xml:space="preserve">CXCL12 </t>
         </is>
       </c>
       <c r="D109" s="38" t="n"/>
@@ -5286,12 +5278,12 @@
       </c>
       <c r="B110" s="32" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>M2R</t>
         </is>
       </c>
       <c r="C110" s="32" t="inlineStr">
         <is>
-          <t>transferrin</t>
+          <t>acetylcholine</t>
         </is>
       </c>
       <c r="D110" s="38" t="n"/>
@@ -5300,19 +5292,19 @@
       <c r="G110" s="38" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="40" t="inlineStr">
-        <is>
-          <t>Kins</t>
+      <c r="A111" s="35" t="inlineStr">
+        <is>
+          <t>Krec</t>
         </is>
       </c>
       <c r="B111" s="32" t="inlineStr">
         <is>
-          <t>α2AR</t>
+          <t>V1R</t>
         </is>
       </c>
       <c r="C111" s="32" t="inlineStr">
         <is>
-          <t>UK14304</t>
+          <t>arginine vasopressin</t>
         </is>
       </c>
       <c r="D111" s="38" t="n"/>
@@ -5321,19 +5313,19 @@
       <c r="G111" s="38" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="40" t="inlineStr">
-        <is>
-          <t>Kins</t>
+      <c r="A112" s="35" t="inlineStr">
+        <is>
+          <t>Krec</t>
         </is>
       </c>
       <c r="B112" s="32" t="inlineStr">
         <is>
-          <t>VSVG-GFP</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C112" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/A </t>
+          <t>transferrin</t>
         </is>
       </c>
       <c r="D112" s="38" t="n"/>
@@ -5349,12 +5341,12 @@
       </c>
       <c r="B113" s="32" t="inlineStr">
         <is>
-          <t>M2R</t>
+          <t>α2AR</t>
         </is>
       </c>
       <c r="C113" s="32" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t>UK14304</t>
         </is>
       </c>
       <c r="D113" s="38" t="n"/>
@@ -5386,17 +5378,17 @@
     <row r="115">
       <c r="A115" s="40" t="inlineStr">
         <is>
-          <t>Krgt</t>
+          <t>Kins</t>
         </is>
       </c>
       <c r="B115" s="32" t="inlineStr">
         <is>
-          <t>VSVG-GFP</t>
+          <t>M2R</t>
         </is>
       </c>
       <c r="C115" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/A </t>
+          <t>acetylcholine</t>
         </is>
       </c>
       <c r="D115" s="38" t="n"/>
@@ -5407,12 +5399,12 @@
     <row r="116">
       <c r="A116" s="40" t="inlineStr">
         <is>
-          <t>Krgt</t>
+          <t>Kins</t>
         </is>
       </c>
       <c r="B116" s="32" t="inlineStr">
         <is>
-          <t>INGF</t>
+          <t>VSVG-GFP</t>
         </is>
       </c>
       <c r="C116" s="32" t="inlineStr">
@@ -5454,12 +5446,12 @@
       </c>
       <c r="B118" s="32" t="inlineStr">
         <is>
-          <t>EGFP-CDMPR</t>
+          <t>INGF</t>
         </is>
       </c>
       <c r="C118" s="32" t="inlineStr">
         <is>
-          <t>mannose-6-phosphate (M6P)</t>
+          <t xml:space="preserve">N/A </t>
         </is>
       </c>
       <c r="D118" s="38" t="n"/>
@@ -5475,12 +5467,12 @@
       </c>
       <c r="B119" s="32" t="inlineStr">
         <is>
-          <t>EGFP-CDMPR</t>
+          <t>VSVG-GFP</t>
         </is>
       </c>
       <c r="C119" s="32" t="inlineStr">
         <is>
-          <t>mannose-6-phosphate (M6P)</t>
+          <t xml:space="preserve">N/A </t>
         </is>
       </c>
       <c r="D119" s="38" t="n"/>
@@ -5533,17 +5525,17 @@
     <row r="122">
       <c r="A122" s="40" t="inlineStr">
         <is>
-          <t>Kdeg</t>
+          <t>Krgt</t>
         </is>
       </c>
       <c r="B122" s="32" t="inlineStr">
         <is>
-          <t>α1AR</t>
+          <t>EGFP-CDMPR</t>
         </is>
       </c>
       <c r="C122" s="32" t="inlineStr">
         <is>
-          <t>phenylephrine</t>
+          <t>mannose-6-phosphate (M6P)</t>
         </is>
       </c>
       <c r="D122" s="38" t="n"/>
@@ -5554,17 +5546,17 @@
     <row r="123">
       <c r="A123" s="40" t="inlineStr">
         <is>
-          <t>Kdeg</t>
+          <t>Krgt</t>
         </is>
       </c>
       <c r="B123" s="32" t="inlineStr">
         <is>
-          <t>α2AR</t>
+          <t>EGFP-CDMPR</t>
         </is>
       </c>
       <c r="C123" s="32" t="inlineStr">
         <is>
-          <t>phenylephrine</t>
+          <t>mannose-6-phosphate (M6P)</t>
         </is>
       </c>
       <c r="D123" s="38" t="n"/>
@@ -5580,12 +5572,12 @@
       </c>
       <c r="B124" s="32" t="inlineStr">
         <is>
-          <t>βXAR</t>
+          <t>α1AR</t>
         </is>
       </c>
       <c r="C124" s="32" t="inlineStr">
         <is>
-          <t>norepinephrine</t>
+          <t>phenylephrine</t>
         </is>
       </c>
       <c r="D124" s="38" t="n"/>
@@ -5601,12 +5593,12 @@
       </c>
       <c r="B125" s="32" t="inlineStr">
         <is>
-          <t>5-HTX</t>
+          <t>α2AR</t>
         </is>
       </c>
       <c r="C125" s="32" t="inlineStr">
         <is>
-          <t>serotonin</t>
+          <t>phenylephrine</t>
         </is>
       </c>
       <c r="D125" s="38" t="n"/>
@@ -5622,12 +5614,12 @@
       </c>
       <c r="B126" s="32" t="inlineStr">
         <is>
-          <t>SSTR</t>
+          <t>βXAR</t>
         </is>
       </c>
       <c r="C126" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/A </t>
+          <t>norepinephrine</t>
         </is>
       </c>
       <c r="D126" s="38" t="n"/>
@@ -5643,12 +5635,12 @@
       </c>
       <c r="B127" s="32" t="inlineStr">
         <is>
-          <t>CXCR</t>
-        </is>
-      </c>
-      <c r="C127" s="34" t="inlineStr">
-        <is>
-          <t>CCL5/CXCL12</t>
+          <t>5-HTX</t>
+        </is>
+      </c>
+      <c r="C127" s="32" t="inlineStr">
+        <is>
+          <t>serotonin</t>
         </is>
       </c>
       <c r="D127" s="38" t="n"/>
@@ -5664,12 +5656,12 @@
       </c>
       <c r="B128" s="32" t="inlineStr">
         <is>
-          <t>AChR</t>
+          <t>SSTR</t>
         </is>
       </c>
       <c r="C128" s="32" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t xml:space="preserve">N/A </t>
         </is>
       </c>
       <c r="D128" s="38" t="n"/>
@@ -5685,12 +5677,12 @@
       </c>
       <c r="B129" s="32" t="inlineStr">
         <is>
-          <t>AChR</t>
-        </is>
-      </c>
-      <c r="C129" s="32" t="inlineStr">
-        <is>
-          <t>acetylcholine</t>
+          <t>CXCR</t>
+        </is>
+      </c>
+      <c r="C129" s="34" t="inlineStr">
+        <is>
+          <t>CCL5/CXCL12</t>
         </is>
       </c>
       <c r="D129" s="38" t="n"/>
@@ -5706,12 +5698,12 @@
       </c>
       <c r="B130" s="32" t="inlineStr">
         <is>
-          <t>5-HT1A</t>
+          <t>AChR</t>
         </is>
       </c>
       <c r="C130" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EEDQ, or N-ethoxycarbonyl-2-ethoxy-1,2-dihydroquinoline </t>
+          <t>acetylcholine</t>
         </is>
       </c>
       <c r="D130" s="38" t="n"/>
@@ -5727,12 +5719,12 @@
       </c>
       <c r="B131" s="32" t="inlineStr">
         <is>
-          <t>5-HT2A</t>
+          <t>AChR</t>
         </is>
       </c>
       <c r="C131" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EEDQ, or N-ethoxycarbonyl-2-ethoxy-1,2-dihydroquinoline </t>
+          <t>acetylcholine</t>
         </is>
       </c>
       <c r="D131" s="38" t="n"/>
@@ -5748,12 +5740,12 @@
       </c>
       <c r="B132" s="32" t="inlineStr">
         <is>
-          <t>β2AR</t>
+          <t>5-HT1A</t>
         </is>
       </c>
       <c r="C132" s="32" t="inlineStr">
         <is>
-          <t>isoproterenol</t>
+          <t xml:space="preserve">EEDQ, or N-ethoxycarbonyl-2-ethoxy-1,2-dihydroquinoline </t>
         </is>
       </c>
       <c r="D132" s="38" t="n"/>
@@ -5769,12 +5761,12 @@
       </c>
       <c r="B133" s="32" t="inlineStr">
         <is>
-          <t>AChR</t>
+          <t>5-HT2A</t>
         </is>
       </c>
       <c r="C133" s="32" t="inlineStr">
         <is>
-          <t>acetylcholine</t>
+          <t xml:space="preserve">EEDQ, or N-ethoxycarbonyl-2-ethoxy-1,2-dihydroquinoline </t>
         </is>
       </c>
       <c r="D133" s="38" t="n"/>
@@ -5790,12 +5782,12 @@
       </c>
       <c r="B134" s="32" t="inlineStr">
         <is>
-          <t>VSVG-GFP</t>
+          <t>β2AR</t>
         </is>
       </c>
       <c r="C134" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/A </t>
+          <t>isoproterenol</t>
         </is>
       </c>
       <c r="D134" s="38" t="n"/>
@@ -5804,23 +5796,65 @@
       <c r="G134" s="38" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="38" t="n"/>
-      <c r="B135" s="38" t="n"/>
-      <c r="C135" s="38" t="n"/>
+      <c r="A135" s="40" t="inlineStr">
+        <is>
+          <t>Kdeg</t>
+        </is>
+      </c>
+      <c r="B135" s="32" t="inlineStr">
+        <is>
+          <t>AChR</t>
+        </is>
+      </c>
+      <c r="C135" s="32" t="inlineStr">
+        <is>
+          <t>acetylcholine</t>
+        </is>
+      </c>
       <c r="D135" s="38" t="n"/>
       <c r="E135" s="38" t="n"/>
       <c r="F135" s="38" t="n"/>
       <c r="G135" s="38" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="38" t="n"/>
-      <c r="B136" s="38" t="n"/>
-      <c r="C136" s="38" t="n"/>
+      <c r="A136" s="40" t="inlineStr">
+        <is>
+          <t>Kdeg</t>
+        </is>
+      </c>
+      <c r="B136" s="32" t="inlineStr">
+        <is>
+          <t>VSVG-GFP</t>
+        </is>
+      </c>
+      <c r="C136" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A </t>
+        </is>
+      </c>
       <c r="D136" s="38" t="n"/>
       <c r="E136" s="38" t="n"/>
       <c r="F136" s="38" t="n"/>
       <c r="G136" s="38" t="n"/>
     </row>
+    <row r="137">
+      <c r="A137" s="38" t="n"/>
+      <c r="B137" s="38" t="n"/>
+      <c r="C137" s="38" t="n"/>
+      <c r="D137" s="38" t="n"/>
+      <c r="E137" s="38" t="n"/>
+      <c r="F137" s="38" t="n"/>
+      <c r="G137" s="38" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="38" t="n"/>
+      <c r="B138" s="38" t="n"/>
+      <c r="C138" s="38" t="n"/>
+      <c r="D138" s="38" t="n"/>
+      <c r="E138" s="38" t="n"/>
+      <c r="F138" s="38" t="n"/>
+      <c r="G138" s="38" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>